<commit_message>
Align Viewpoints tables and setup paths
Update the manuscript table outputs and make the setup path handling portable so collaborators can run the pipeline from a supplied project root.
</commit_message>
<xml_diff>
--- a/output/tables/Table_Viewpoints_Sample_Characteristics.xlsx
+++ b/output/tables/Table_Viewpoints_Sample_Characteristics.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="59" uniqueCount="44">
   <si>
-    <t>Table 2. Sample characteristics, n=1000 AI personas and n=1012 human participants</t>
+    <t>Table 2. Sample characteristics, n=1,000 AI personas and n=1,012 human participants</t>
   </si>
   <si>
     <t>Characteristic</t>
@@ -66,7 +66,7 @@
     <t>492</t>
   </si>
   <si>
-    <t xml:space="preserve">   Non-binary/Other</t>
+    <t xml:space="preserve">   Non-binary/preferred-to-self-describe</t>
   </si>
   <si>
     <t>NA</t>
@@ -78,7 +78,7 @@
     <t>1%</t>
   </si>
   <si>
-    <t>Race or ethnicity</t>
+    <t>Race/ethnicity</t>
   </si>
   <si>
     <t xml:space="preserve">   American Indian/Alaska Native</t>
@@ -141,10 +141,10 @@
     <t>9%</t>
   </si>
   <si>
-    <t>Note. AI personas could only be assigned a gender of female or male, so no personas were assigned to non-binary or another gender identity.</t>
-  </si>
-  <si>
-    <t>AI personas could only be assigned one race/ethnicity from a fixed list of options, so no personas were assigned to American Indian or Alaska Native, Native Hawaiian or Pacific Islander, another race or ethnicity, or multiracial/ethnic.</t>
+    <t>Note. AI personas could only be assigned a gender of female or male, so no personas were assigned to non-binary/preferred-to-self-describe.</t>
+  </si>
+  <si>
+    <t>AI personas could only be assigned one race/ethnicity from a fixed list of options, so no personas were assigned to American Indian/Alaska Native, Native Hawaiian/Pacific Islander, another race/ethnicity, or multiracial/ethnic.</t>
   </si>
 </sst>
 </file>

</xml_diff>